<commit_message>
Update Nalco PDF (2026-09-06 08:01:09 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1285"/>
+  <dimension ref="A1:H1286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -41933,6 +41933,38 @@
       </c>
       <c r="H1285" s="1" t="inlineStr"/>
     </row>
+    <row r="1286">
+      <c r="A1286" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 08:01:04 UTC</t>
+        </is>
+      </c>
+      <c r="B1286" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:31:04 IST</t>
+        </is>
+      </c>
+      <c r="C1286" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1286" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1286" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1286" s="1" t="inlineStr"/>
+      <c r="G1286" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1286" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-06 13:00:21 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1286"/>
+  <dimension ref="A1:H1287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -41965,6 +41965,38 @@
       </c>
       <c r="H1286" s="1" t="inlineStr"/>
     </row>
+    <row r="1287">
+      <c r="A1287" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:00:17 UTC</t>
+        </is>
+      </c>
+      <c r="B1287" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 18:30:17 IST</t>
+        </is>
+      </c>
+      <c r="C1287" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1287" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1287" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1287" s="1" t="inlineStr"/>
+      <c r="G1287" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1287" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-07 08:31:33 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1287"/>
+  <dimension ref="A1:H1288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -41997,6 +41997,38 @@
       </c>
       <c r="H1287" s="1" t="inlineStr"/>
     </row>
+    <row r="1288">
+      <c r="A1288" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07 08:31:28 UTC</t>
+        </is>
+      </c>
+      <c r="B1288" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07 14:01:28 IST</t>
+        </is>
+      </c>
+      <c r="C1288" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1288" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1288" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1288" s="1" t="inlineStr"/>
+      <c r="G1288" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1288" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-07 15:07:57 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1288"/>
+  <dimension ref="A1:H1289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42029,6 +42029,38 @@
       </c>
       <c r="H1288" s="1" t="inlineStr"/>
     </row>
+    <row r="1289">
+      <c r="A1289" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07 15:07:53 UTC</t>
+        </is>
+      </c>
+      <c r="B1289" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07 20:37:53 IST</t>
+        </is>
+      </c>
+      <c r="C1289" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1289" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1289" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1289" s="1" t="inlineStr"/>
+      <c r="G1289" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1289" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-08 13:45:10 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1290"/>
+  <dimension ref="A1:H1291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42099,6 +42099,38 @@
         <v>69</v>
       </c>
     </row>
+    <row r="1291">
+      <c r="A1291" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08 13:45:05 UTC</t>
+        </is>
+      </c>
+      <c r="B1291" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08 19:15:05 IST</t>
+        </is>
+      </c>
+      <c r="C1291" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1291" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1291" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1291" s="1" t="inlineStr"/>
+      <c r="G1291" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1291" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-09 08:17:24 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1291"/>
+  <dimension ref="A1:H1292"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42131,6 +42131,38 @@
       </c>
       <c r="H1291" s="1" t="inlineStr"/>
     </row>
+    <row r="1292">
+      <c r="A1292" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09 08:17:19 UTC</t>
+        </is>
+      </c>
+      <c r="B1292" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:47:19 IST</t>
+        </is>
+      </c>
+      <c r="C1292" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1292" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1292" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1292" s="1" t="inlineStr"/>
+      <c r="G1292" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1292" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-11 11:06:55 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1293"/>
+  <dimension ref="A1:H1294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42201,6 +42201,38 @@
         <v>70</v>
       </c>
     </row>
+    <row r="1294">
+      <c r="A1294" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-11 11:06:51 UTC</t>
+        </is>
+      </c>
+      <c r="B1294" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-11 16:36:51 IST</t>
+        </is>
+      </c>
+      <c r="C1294" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1294" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1294" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1294" s="1" t="inlineStr"/>
+      <c r="G1294" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1294" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-11 13:41:35 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1294"/>
+  <dimension ref="A1:H1295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42233,6 +42233,38 @@
       </c>
       <c r="H1294" s="1" t="inlineStr"/>
     </row>
+    <row r="1295">
+      <c r="A1295" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:41:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1295" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-11 19:11:30 IST</t>
+        </is>
+      </c>
+      <c r="C1295" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1295" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1295" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1295" s="1" t="inlineStr"/>
+      <c r="G1295" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1295" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-12 08:02:10 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1295"/>
+  <dimension ref="A1:H1296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42265,6 +42265,38 @@
       </c>
       <c r="H1295" s="1" t="inlineStr"/>
     </row>
+    <row r="1296">
+      <c r="A1296" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-12 08:02:05 UTC</t>
+        </is>
+      </c>
+      <c r="B1296" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-12 13:32:05 IST</t>
+        </is>
+      </c>
+      <c r="C1296" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1296" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1296" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1296" s="1" t="inlineStr"/>
+      <c r="G1296" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1296" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-12 12:57:48 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1296"/>
+  <dimension ref="A1:H1297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42297,6 +42297,38 @@
       </c>
       <c r="H1296" s="1" t="inlineStr"/>
     </row>
+    <row r="1297">
+      <c r="A1297" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-12 12:57:43 UTC</t>
+        </is>
+      </c>
+      <c r="B1297" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-12 18:27:43 IST</t>
+        </is>
+      </c>
+      <c r="C1297" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1297" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1297" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1297" s="1" t="inlineStr"/>
+      <c r="G1297" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1297" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-13 08:27:01 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1297"/>
+  <dimension ref="A1:H1298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42329,6 +42329,38 @@
       </c>
       <c r="H1297" s="1" t="inlineStr"/>
     </row>
+    <row r="1298">
+      <c r="A1298" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-13 08:26:57 UTC</t>
+        </is>
+      </c>
+      <c r="B1298" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:56:57 IST</t>
+        </is>
+      </c>
+      <c r="C1298" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1298" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1298" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1298" s="1" t="inlineStr"/>
+      <c r="G1298" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1298" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-13 13:50:49 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1298"/>
+  <dimension ref="A1:H1299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42361,6 +42361,38 @@
       </c>
       <c r="H1298" s="1" t="inlineStr"/>
     </row>
+    <row r="1299">
+      <c r="A1299" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:50:45 UTC</t>
+        </is>
+      </c>
+      <c r="B1299" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-13 19:20:45 IST</t>
+        </is>
+      </c>
+      <c r="C1299" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1299" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1299" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1299" s="1" t="inlineStr"/>
+      <c r="G1299" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1299" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-14 09:08:24 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1299"/>
+  <dimension ref="A1:H1300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42393,6 +42393,38 @@
       </c>
       <c r="H1299" s="1" t="inlineStr"/>
     </row>
+    <row r="1300">
+      <c r="A1300" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-14 09:08:19 UTC</t>
+        </is>
+      </c>
+      <c r="B1300" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-14 14:38:19 IST</t>
+        </is>
+      </c>
+      <c r="C1300" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1300" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1300" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1300" s="1" t="inlineStr"/>
+      <c r="G1300" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1300" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-14 15:57:04 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1300"/>
+  <dimension ref="A1:H1301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42425,6 +42425,38 @@
       </c>
       <c r="H1300" s="1" t="inlineStr"/>
     </row>
+    <row r="1301">
+      <c r="A1301" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-14 15:57:00 UTC</t>
+        </is>
+      </c>
+      <c r="B1301" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-14 21:27:00 IST</t>
+        </is>
+      </c>
+      <c r="C1301" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1301" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1301" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1301" s="1" t="inlineStr"/>
+      <c r="G1301" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1301" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-15 08:50:27 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1301"/>
+  <dimension ref="A1:H1302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42457,6 +42457,38 @@
       </c>
       <c r="H1301" s="1" t="inlineStr"/>
     </row>
+    <row r="1302">
+      <c r="A1302" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15 08:50:21 UTC</t>
+        </is>
+      </c>
+      <c r="B1302" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15 14:20:21 IST</t>
+        </is>
+      </c>
+      <c r="C1302" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1302" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1302" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1302" s="1" t="inlineStr"/>
+      <c r="G1302" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1302" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-15 14:23:08 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1302"/>
+  <dimension ref="A1:H1303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42489,6 +42489,38 @@
       </c>
       <c r="H1302" s="1" t="inlineStr"/>
     </row>
+    <row r="1303">
+      <c r="A1303" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15 14:23:05 UTC</t>
+        </is>
+      </c>
+      <c r="B1303" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15 19:53:05 IST</t>
+        </is>
+      </c>
+      <c r="C1303" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1303" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1303" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1303" s="1" t="inlineStr"/>
+      <c r="G1303" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1303" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-16 14:15:55 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1304"/>
+  <dimension ref="A1:H1305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42559,6 +42559,38 @@
         <v>71</v>
       </c>
     </row>
+    <row r="1305">
+      <c r="A1305" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-16 14:15:51 UTC</t>
+        </is>
+      </c>
+      <c r="B1305" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-16 19:45:51 IST</t>
+        </is>
+      </c>
+      <c r="C1305" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1305" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1305" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1305" s="1" t="inlineStr"/>
+      <c r="G1305" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1305" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-17 08:48:04 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1305"/>
+  <dimension ref="A1:H1306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42591,6 +42591,38 @@
       </c>
       <c r="H1305" s="1" t="inlineStr"/>
     </row>
+    <row r="1306">
+      <c r="A1306" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17 08:47:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1306" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:17:59 IST</t>
+        </is>
+      </c>
+      <c r="C1306" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1306" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1306" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1306" s="1" t="inlineStr"/>
+      <c r="G1306" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1306" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-17 14:21:57 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1306"/>
+  <dimension ref="A1:H1307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42623,6 +42623,38 @@
       </c>
       <c r="H1306" s="1" t="inlineStr"/>
     </row>
+    <row r="1307">
+      <c r="A1307" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:21:52 UTC</t>
+        </is>
+      </c>
+      <c r="B1307" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17 19:51:52 IST</t>
+        </is>
+      </c>
+      <c r="C1307" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1307" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1307" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1307" s="1" t="inlineStr"/>
+      <c r="G1307" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1307" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-18 08:23:51 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1307"/>
+  <dimension ref="A1:H1308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42655,6 +42655,38 @@
       </c>
       <c r="H1307" s="1" t="inlineStr"/>
     </row>
+    <row r="1308">
+      <c r="A1308" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-18 08:23:47 UTC</t>
+        </is>
+      </c>
+      <c r="B1308" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:53:47 IST</t>
+        </is>
+      </c>
+      <c r="C1308" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1308" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1308" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1308" s="1" t="inlineStr"/>
+      <c r="G1308" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1308" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-18 13:42:12 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1308"/>
+  <dimension ref="A1:H1309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42687,6 +42687,38 @@
       </c>
       <c r="H1308" s="1" t="inlineStr"/>
     </row>
+    <row r="1309">
+      <c r="A1309" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:42:08 UTC</t>
+        </is>
+      </c>
+      <c r="B1309" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-18 19:12:08 IST</t>
+        </is>
+      </c>
+      <c r="C1309" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1309" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1309" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1309" s="1" t="inlineStr"/>
+      <c r="G1309" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1309" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-19 13:15:30 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1310"/>
+  <dimension ref="A1:H1311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42757,6 +42757,38 @@
         <v>72</v>
       </c>
     </row>
+    <row r="1311">
+      <c r="A1311" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-19 13:15:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1311" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-19 18:45:25 IST</t>
+        </is>
+      </c>
+      <c r="C1311" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1311" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1311" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1311" s="1" t="inlineStr"/>
+      <c r="G1311" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1311" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-20 08:43:49 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1311"/>
+  <dimension ref="A1:H1312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42789,6 +42789,38 @@
       </c>
       <c r="H1311" s="1" t="inlineStr"/>
     </row>
+    <row r="1312">
+      <c r="A1312" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-20 08:43:46 UTC</t>
+        </is>
+      </c>
+      <c r="B1312" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-20 14:13:46 IST</t>
+        </is>
+      </c>
+      <c r="C1312" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1312" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1312" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1312" s="1" t="inlineStr"/>
+      <c r="G1312" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1312" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-20 13:38:02 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1312"/>
+  <dimension ref="A1:H1313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42821,6 +42821,38 @@
       </c>
       <c r="H1312" s="1" t="inlineStr"/>
     </row>
+    <row r="1313">
+      <c r="A1313" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-20 13:37:58 UTC</t>
+        </is>
+      </c>
+      <c r="B1313" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-20 19:07:58 IST</t>
+        </is>
+      </c>
+      <c r="C1313" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1313" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1313" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1313" s="1" t="inlineStr"/>
+      <c r="G1313" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1313" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-21 09:10:27 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1313"/>
+  <dimension ref="A1:H1314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42853,6 +42853,38 @@
       </c>
       <c r="H1313" s="1" t="inlineStr"/>
     </row>
+    <row r="1314">
+      <c r="A1314" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-21 09:10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B1314" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-21 14:40:23 IST</t>
+        </is>
+      </c>
+      <c r="C1314" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1314" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1314" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1314" s="1" t="inlineStr"/>
+      <c r="G1314" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1314" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-21 15:58:09 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1314"/>
+  <dimension ref="A1:H1315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42885,6 +42885,38 @@
       </c>
       <c r="H1314" s="1" t="inlineStr"/>
     </row>
+    <row r="1315">
+      <c r="A1315" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:58:04 UTC</t>
+        </is>
+      </c>
+      <c r="B1315" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-21 21:28:04 IST</t>
+        </is>
+      </c>
+      <c r="C1315" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1315" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1315" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1315" s="1" t="inlineStr"/>
+      <c r="G1315" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1315" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-22 08:41:56 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1315"/>
+  <dimension ref="A1:H1316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42917,6 +42917,38 @@
       </c>
       <c r="H1315" s="1" t="inlineStr"/>
     </row>
+    <row r="1316">
+      <c r="A1316" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-22 08:41:51 UTC</t>
+        </is>
+      </c>
+      <c r="B1316" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:11:51 IST</t>
+        </is>
+      </c>
+      <c r="C1316" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1316" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1316" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1316" s="1" t="inlineStr"/>
+      <c r="G1316" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1316" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-22 14:05:54 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1316"/>
+  <dimension ref="A1:H1317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42949,6 +42949,38 @@
       </c>
       <c r="H1316" s="1" t="inlineStr"/>
     </row>
+    <row r="1317">
+      <c r="A1317" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:05:49 UTC</t>
+        </is>
+      </c>
+      <c r="B1317" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-22 19:35:49 IST</t>
+        </is>
+      </c>
+      <c r="C1317" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1317" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1317" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1317" s="1" t="inlineStr"/>
+      <c r="G1317" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1317" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-23 08:44:08 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1317"/>
+  <dimension ref="A1:H1318"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -42981,6 +42981,38 @@
       </c>
       <c r="H1317" s="1" t="inlineStr"/>
     </row>
+    <row r="1318">
+      <c r="A1318" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:44:02 UTC</t>
+        </is>
+      </c>
+      <c r="B1318" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-23 14:14:02 IST</t>
+        </is>
+      </c>
+      <c r="C1318" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1318" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1318" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1318" s="1" t="inlineStr"/>
+      <c r="G1318" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1318" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-23 14:18:08 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1318"/>
+  <dimension ref="A1:H1319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43013,6 +43013,38 @@
       </c>
       <c r="H1318" s="1" t="inlineStr"/>
     </row>
+    <row r="1319">
+      <c r="A1319" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-23 14:18:05 UTC</t>
+        </is>
+      </c>
+      <c r="B1319" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-23 19:48:05 IST</t>
+        </is>
+      </c>
+      <c r="C1319" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1319" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1319" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1319" s="1" t="inlineStr"/>
+      <c r="G1319" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1319" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-24 14:16:41 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1320"/>
+  <dimension ref="A1:H1321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43083,6 +43083,38 @@
         <v>73</v>
       </c>
     </row>
+    <row r="1321">
+      <c r="A1321" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:16:37 UTC</t>
+        </is>
+      </c>
+      <c r="B1321" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-24 19:46:37 IST</t>
+        </is>
+      </c>
+      <c r="C1321" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1321" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1321" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1321" s="1" t="inlineStr"/>
+      <c r="G1321" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1321" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-25 08:58:43 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1321"/>
+  <dimension ref="A1:H1322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43115,6 +43115,38 @@
       </c>
       <c r="H1321" s="1" t="inlineStr"/>
     </row>
+    <row r="1322">
+      <c r="A1322" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-25 08:58:39 UTC</t>
+        </is>
+      </c>
+      <c r="B1322" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:28:39 IST</t>
+        </is>
+      </c>
+      <c r="C1322" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1322" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1322" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1322" s="1" t="inlineStr"/>
+      <c r="G1322" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1322" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-25 14:40:04 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1322"/>
+  <dimension ref="A1:H1323"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43147,6 +43147,38 @@
       </c>
       <c r="H1322" s="1" t="inlineStr"/>
     </row>
+    <row r="1323">
+      <c r="A1323" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:39:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1323" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-25 20:09:59 IST</t>
+        </is>
+      </c>
+      <c r="C1323" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1323" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1323" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1323" s="1" t="inlineStr"/>
+      <c r="G1323" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1323" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-26 08:44:51 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1323"/>
+  <dimension ref="A1:H1324"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43179,6 +43179,38 @@
       </c>
       <c r="H1323" s="1" t="inlineStr"/>
     </row>
+    <row r="1324">
+      <c r="A1324" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-26 08:44:47 UTC</t>
+        </is>
+      </c>
+      <c r="B1324" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-26 14:14:47 IST</t>
+        </is>
+      </c>
+      <c r="C1324" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1324" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1324" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1324" s="1" t="inlineStr"/>
+      <c r="G1324" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1324" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-26 13:48:00 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1324"/>
+  <dimension ref="A1:H1325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43211,6 +43211,38 @@
       </c>
       <c r="H1324" s="1" t="inlineStr"/>
     </row>
+    <row r="1325">
+      <c r="A1325" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:47:55 UTC</t>
+        </is>
+      </c>
+      <c r="B1325" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-26 19:17:55 IST</t>
+        </is>
+      </c>
+      <c r="C1325" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1325" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1325" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1325" s="1" t="inlineStr"/>
+      <c r="G1325" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1325" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-27 09:25:13 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1325"/>
+  <dimension ref="A1:H1326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43243,6 +43243,38 @@
       </c>
       <c r="H1325" s="1" t="inlineStr"/>
     </row>
+    <row r="1326">
+      <c r="A1326" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-27 09:25:09 UTC</t>
+        </is>
+      </c>
+      <c r="B1326" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:55:09 IST</t>
+        </is>
+      </c>
+      <c r="C1326" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1326" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1326" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1326" s="1" t="inlineStr"/>
+      <c r="G1326" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1326" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-27 14:45:54 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1326"/>
+  <dimension ref="A1:H1327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43275,6 +43275,38 @@
       </c>
       <c r="H1326" s="1" t="inlineStr"/>
     </row>
+    <row r="1327">
+      <c r="A1327" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:45:49 UTC</t>
+        </is>
+      </c>
+      <c r="B1327" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-27 20:15:49 IST</t>
+        </is>
+      </c>
+      <c r="C1327" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1327" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1327" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1327" s="1" t="inlineStr"/>
+      <c r="G1327" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1327" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-28 10:01:56 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1327"/>
+  <dimension ref="A1:H1328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43307,6 +43307,38 @@
       </c>
       <c r="H1327" s="1" t="inlineStr"/>
     </row>
+    <row r="1328">
+      <c r="A1328" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-28 10:01:51 UTC</t>
+        </is>
+      </c>
+      <c r="B1328" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:31:51 IST</t>
+        </is>
+      </c>
+      <c r="C1328" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1328" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1328" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1328" s="1" t="inlineStr"/>
+      <c r="G1328" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1328" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-28 19:45:45 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1328"/>
+  <dimension ref="A1:H1329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43339,6 +43339,38 @@
       </c>
       <c r="H1328" s="1" t="inlineStr"/>
     </row>
+    <row r="1329">
+      <c r="A1329" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:45:41 UTC</t>
+        </is>
+      </c>
+      <c r="B1329" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-29 01:15:41 IST</t>
+        </is>
+      </c>
+      <c r="C1329" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1329" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1329" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1329" s="1" t="inlineStr"/>
+      <c r="G1329" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1329" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-29 10:00:54 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1329"/>
+  <dimension ref="A1:H1330"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43371,6 +43371,38 @@
       </c>
       <c r="H1329" s="1" t="inlineStr"/>
     </row>
+    <row r="1330">
+      <c r="A1330" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:00:49 UTC</t>
+        </is>
+      </c>
+      <c r="B1330" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:30:49 IST</t>
+        </is>
+      </c>
+      <c r="C1330" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1330" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1330" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1330" s="1" t="inlineStr"/>
+      <c r="G1330" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1330" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-29 18:10:29 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1330"/>
+  <dimension ref="A1:H1331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43403,6 +43403,38 @@
       </c>
       <c r="H1330" s="1" t="inlineStr"/>
     </row>
+    <row r="1331">
+      <c r="A1331" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-29 18:10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B1331" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-29 23:40:23 IST</t>
+        </is>
+      </c>
+      <c r="C1331" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1331" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1331" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1331" s="1" t="inlineStr"/>
+      <c r="G1331" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1331" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-30 09:53:16 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1331"/>
+  <dimension ref="A1:H1332"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43435,6 +43435,38 @@
       </c>
       <c r="H1331" s="1" t="inlineStr"/>
     </row>
+    <row r="1332">
+      <c r="A1332" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-30 09:53:11 UTC</t>
+        </is>
+      </c>
+      <c r="B1332" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-30 15:23:11 IST</t>
+        </is>
+      </c>
+      <c r="C1332" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1332" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1332" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1332" s="1" t="inlineStr"/>
+      <c r="G1332" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1332" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-30 18:02:57 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1332"/>
+  <dimension ref="A1:H1333"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43467,6 +43467,38 @@
       </c>
       <c r="H1332" s="1" t="inlineStr"/>
     </row>
+    <row r="1333">
+      <c r="A1333" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-30 18:02:53 UTC</t>
+        </is>
+      </c>
+      <c r="B1333" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:32:53 IST</t>
+        </is>
+      </c>
+      <c r="C1333" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1333" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1333" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1333" s="1" t="inlineStr"/>
+      <c r="G1333" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1333" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-01 10:20:23 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1333"/>
+  <dimension ref="A1:H1334"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43499,6 +43499,38 @@
       </c>
       <c r="H1333" s="1" t="inlineStr"/>
     </row>
+    <row r="1334">
+      <c r="A1334" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-01 10:20:18 UTC</t>
+        </is>
+      </c>
+      <c r="B1334" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-01 15:50:18 IST</t>
+        </is>
+      </c>
+      <c r="C1334" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1334" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1334" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1334" s="1" t="inlineStr"/>
+      <c r="G1334" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1334" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-01 18:29:45 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1334"/>
+  <dimension ref="A1:H1335"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43531,6 +43531,38 @@
       </c>
       <c r="H1334" s="1" t="inlineStr"/>
     </row>
+    <row r="1335">
+      <c r="A1335" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-01 18:29:40 UTC</t>
+        </is>
+      </c>
+      <c r="B1335" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-01 23:59:40 IST</t>
+        </is>
+      </c>
+      <c r="C1335" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1335" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1335" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1335" s="1" t="inlineStr"/>
+      <c r="G1335" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1335" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-02 17:56:57 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1336"/>
+  <dimension ref="A1:H1337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43601,6 +43601,38 @@
         <v>74</v>
       </c>
     </row>
+    <row r="1337">
+      <c r="A1337" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-02 17:56:52 UTC</t>
+        </is>
+      </c>
+      <c r="B1337" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-02 23:26:52 IST</t>
+        </is>
+      </c>
+      <c r="C1337" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1337" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1337" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1337" s="1" t="inlineStr"/>
+      <c r="G1337" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1337" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-03 09:19:24 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1337"/>
+  <dimension ref="A1:H1338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43633,6 +43633,38 @@
       </c>
       <c r="H1337" s="1" t="inlineStr"/>
     </row>
+    <row r="1338">
+      <c r="A1338" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-03 09:19:20 UTC</t>
+        </is>
+      </c>
+      <c r="B1338" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:49:20 IST</t>
+        </is>
+      </c>
+      <c r="C1338" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1338" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1338" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1338" s="1" t="inlineStr"/>
+      <c r="G1338" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1338" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-03 14:21:59 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1338"/>
+  <dimension ref="A1:H1339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43665,6 +43665,38 @@
       </c>
       <c r="H1338" s="1" t="inlineStr"/>
     </row>
+    <row r="1339">
+      <c r="A1339" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:21:55 UTC</t>
+        </is>
+      </c>
+      <c r="B1339" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-03 19:51:55 IST</t>
+        </is>
+      </c>
+      <c r="C1339" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1339" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1339" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1339" s="1" t="inlineStr"/>
+      <c r="G1339" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1339" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-04 09:58:58 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1339"/>
+  <dimension ref="A1:H1340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43697,6 +43697,38 @@
       </c>
       <c r="H1339" s="1" t="inlineStr"/>
     </row>
+    <row r="1340">
+      <c r="A1340" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-04 09:58:52 UTC</t>
+        </is>
+      </c>
+      <c r="B1340" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-04 15:28:52 IST</t>
+        </is>
+      </c>
+      <c r="C1340" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1340" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1340" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1340" s="1" t="inlineStr"/>
+      <c r="G1340" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1340" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-04 16:55:09 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1340"/>
+  <dimension ref="A1:H1341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43729,6 +43729,38 @@
       </c>
       <c r="H1340" s="1" t="inlineStr"/>
     </row>
+    <row r="1341">
+      <c r="A1341" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-04 16:55:05 UTC</t>
+        </is>
+      </c>
+      <c r="B1341" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-04 22:25:05 IST</t>
+        </is>
+      </c>
+      <c r="C1341" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1341" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1341" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1341" s="1" t="inlineStr"/>
+      <c r="G1341" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1341" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-05 10:42:46 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1341"/>
+  <dimension ref="A1:H1342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43761,6 +43761,38 @@
       </c>
       <c r="H1341" s="1" t="inlineStr"/>
     </row>
+    <row r="1342">
+      <c r="A1342" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:42:42 UTC</t>
+        </is>
+      </c>
+      <c r="B1342" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-05 16:12:42 IST</t>
+        </is>
+      </c>
+      <c r="C1342" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1342" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1342" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1342" s="1" t="inlineStr"/>
+      <c r="G1342" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1342" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-06 10:35:56 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1342"/>
+  <dimension ref="A1:H1343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43793,6 +43793,38 @@
       </c>
       <c r="H1342" s="1" t="inlineStr"/>
     </row>
+    <row r="1343">
+      <c r="A1343" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-06 10:35:53 UTC</t>
+        </is>
+      </c>
+      <c r="B1343" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:05:53 IST</t>
+        </is>
+      </c>
+      <c r="C1343" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1343" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1343" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1343" s="1" t="inlineStr"/>
+      <c r="G1343" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1343" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-06 18:30:55 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1343"/>
+  <dimension ref="A1:H1344"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43825,6 +43825,38 @@
       </c>
       <c r="H1343" s="1" t="inlineStr"/>
     </row>
+    <row r="1344">
+      <c r="A1344" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-06 18:30:52 UTC</t>
+        </is>
+      </c>
+      <c r="B1344" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:00:52 IST</t>
+        </is>
+      </c>
+      <c r="C1344" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1344" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1344" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1344" s="1" t="inlineStr"/>
+      <c r="G1344" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1344" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-07 10:27:19 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1344"/>
+  <dimension ref="A1:H1345"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43857,6 +43857,38 @@
       </c>
       <c r="H1344" s="1" t="inlineStr"/>
     </row>
+    <row r="1345">
+      <c r="A1345" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-07 10:27:14 UTC</t>
+        </is>
+      </c>
+      <c r="B1345" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-07 15:57:14 IST</t>
+        </is>
+      </c>
+      <c r="C1345" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1345" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1345" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1345" s="1" t="inlineStr"/>
+      <c r="G1345" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1345" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-07 19:00:55 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1345"/>
+  <dimension ref="A1:H1346"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43889,6 +43889,38 @@
       </c>
       <c r="H1345" s="1" t="inlineStr"/>
     </row>
+    <row r="1346">
+      <c r="A1346" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-07 19:00:50 UTC</t>
+        </is>
+      </c>
+      <c r="B1346" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-08 00:30:50 IST</t>
+        </is>
+      </c>
+      <c r="C1346" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1346" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1346" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1346" s="1" t="inlineStr"/>
+      <c r="G1346" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1346" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-08 10:48:19 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1346"/>
+  <dimension ref="A1:H1347"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43921,6 +43921,38 @@
       </c>
       <c r="H1346" s="1" t="inlineStr"/>
     </row>
+    <row r="1347">
+      <c r="A1347" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-08 10:48:14 UTC</t>
+        </is>
+      </c>
+      <c r="B1347" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:18:14 IST</t>
+        </is>
+      </c>
+      <c r="C1347" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1347" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1347" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1347" s="1" t="inlineStr"/>
+      <c r="G1347" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1347" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-08 18:56:12 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1347"/>
+  <dimension ref="A1:H1348"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43953,6 +43953,38 @@
       </c>
       <c r="H1347" s="1" t="inlineStr"/>
     </row>
+    <row r="1348">
+      <c r="A1348" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-08 18:56:08 UTC</t>
+        </is>
+      </c>
+      <c r="B1348" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-09 00:26:08 IST</t>
+        </is>
+      </c>
+      <c r="C1348" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1348" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1348" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1348" s="1" t="inlineStr"/>
+      <c r="G1348" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1348" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-09 10:46:47 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1348"/>
+  <dimension ref="A1:H1349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -43985,6 +43985,38 @@
       </c>
       <c r="H1348" s="1" t="inlineStr"/>
     </row>
+    <row r="1349">
+      <c r="A1349" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-09 10:46:42 UTC</t>
+        </is>
+      </c>
+      <c r="B1349" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:16:42 IST</t>
+        </is>
+      </c>
+      <c r="C1349" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1349" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1349" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1349" s="1" t="inlineStr"/>
+      <c r="G1349" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1349" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-09 18:26:41 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1349"/>
+  <dimension ref="A1:H1350"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44017,6 +44017,38 @@
       </c>
       <c r="H1349" s="1" t="inlineStr"/>
     </row>
+    <row r="1350">
+      <c r="A1350" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-09 18:26:36 UTC</t>
+        </is>
+      </c>
+      <c r="B1350" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-09 23:56:36 IST</t>
+        </is>
+      </c>
+      <c r="C1350" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1350" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1350" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1350" s="1" t="inlineStr"/>
+      <c r="G1350" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1350" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-10 10:01:47 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1350"/>
+  <dimension ref="A1:H1351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44049,6 +44049,38 @@
       </c>
       <c r="H1350" s="1" t="inlineStr"/>
     </row>
+    <row r="1351">
+      <c r="A1351" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-10 10:01:43 UTC</t>
+        </is>
+      </c>
+      <c r="B1351" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-10 15:31:43 IST</t>
+        </is>
+      </c>
+      <c r="C1351" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1351" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1351" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1351" s="1" t="inlineStr"/>
+      <c r="G1351" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1351" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-10 17:24:37 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1351"/>
+  <dimension ref="A1:H1352"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44081,6 +44081,38 @@
       </c>
       <c r="H1351" s="1" t="inlineStr"/>
     </row>
+    <row r="1352">
+      <c r="A1352" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-10 17:24:32 UTC</t>
+        </is>
+      </c>
+      <c r="B1352" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-10 22:54:32 IST</t>
+        </is>
+      </c>
+      <c r="C1352" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1352" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1352" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1352" s="1" t="inlineStr"/>
+      <c r="G1352" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1352" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-11 10:12:09 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1352"/>
+  <dimension ref="A1:H1353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44113,6 +44113,38 @@
       </c>
       <c r="H1352" s="1" t="inlineStr"/>
     </row>
+    <row r="1353">
+      <c r="A1353" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-11 10:12:04 UTC</t>
+        </is>
+      </c>
+      <c r="B1353" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:42:04 IST</t>
+        </is>
+      </c>
+      <c r="C1353" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1353" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1353" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1353" s="1" t="inlineStr"/>
+      <c r="G1353" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1353" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-11 17:43:53 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1353"/>
+  <dimension ref="A1:H1354"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44145,6 +44145,38 @@
       </c>
       <c r="H1353" s="1" t="inlineStr"/>
     </row>
+    <row r="1354">
+      <c r="A1354" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-11 17:43:49 UTC</t>
+        </is>
+      </c>
+      <c r="B1354" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-11 23:13:49 IST</t>
+        </is>
+      </c>
+      <c r="C1354" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1354" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1354" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1354" s="1" t="inlineStr"/>
+      <c r="G1354" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1354" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-12 11:10:27 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1354"/>
+  <dimension ref="A1:H1355"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44177,6 +44177,38 @@
       </c>
       <c r="H1354" s="1" t="inlineStr"/>
     </row>
+    <row r="1355">
+      <c r="A1355" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-12 11:10:22 UTC</t>
+        </is>
+      </c>
+      <c r="B1355" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-12 16:40:22 IST</t>
+        </is>
+      </c>
+      <c r="C1355" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1355" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1355" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1355" s="1" t="inlineStr"/>
+      <c r="G1355" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1355" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-12 21:20:36 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1355"/>
+  <dimension ref="A1:H1356"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44209,6 +44209,38 @@
       </c>
       <c r="H1355" s="1" t="inlineStr"/>
     </row>
+    <row r="1356">
+      <c r="A1356" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-12 21:20:31 UTC</t>
+        </is>
+      </c>
+      <c r="B1356" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-13 02:50:31 IST</t>
+        </is>
+      </c>
+      <c r="C1356" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1356" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1356" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1356" s="1" t="inlineStr"/>
+      <c r="G1356" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1356" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-13 19:24:59 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1357"/>
+  <dimension ref="A1:H1358"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44279,6 +44279,38 @@
         <v>75</v>
       </c>
     </row>
+    <row r="1358">
+      <c r="A1358" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-13 19:24:54 UTC</t>
+        </is>
+      </c>
+      <c r="B1358" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:54:54 IST</t>
+        </is>
+      </c>
+      <c r="C1358" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1358" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1358" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1358" s="1" t="inlineStr"/>
+      <c r="G1358" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1358" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-14 08:54:00 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1358"/>
+  <dimension ref="A1:H1359"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44311,6 +44311,38 @@
       </c>
       <c r="H1358" s="1" t="inlineStr"/>
     </row>
+    <row r="1359">
+      <c r="A1359" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-14 08:53:55 UTC</t>
+        </is>
+      </c>
+      <c r="B1359" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:23:55 IST</t>
+        </is>
+      </c>
+      <c r="C1359" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1359" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1359" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1359" s="1" t="inlineStr"/>
+      <c r="G1359" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1359" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-14 14:35:22 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1359"/>
+  <dimension ref="A1:H1360"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44343,6 +44343,38 @@
       </c>
       <c r="H1359" s="1" t="inlineStr"/>
     </row>
+    <row r="1360">
+      <c r="A1360" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:35:17 UTC</t>
+        </is>
+      </c>
+      <c r="B1360" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:05:17 IST</t>
+        </is>
+      </c>
+      <c r="C1360" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1360" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1360" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1360" s="1" t="inlineStr"/>
+      <c r="G1360" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1360" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-15 08:28:59 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1360"/>
+  <dimension ref="A1:H1361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44375,6 +44375,38 @@
       </c>
       <c r="H1360" s="1" t="inlineStr"/>
     </row>
+    <row r="1361">
+      <c r="A1361" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-15 08:28:54 UTC</t>
+        </is>
+      </c>
+      <c r="B1361" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-15 13:58:54 IST</t>
+        </is>
+      </c>
+      <c r="C1361" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1361" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1361" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1361" s="1" t="inlineStr"/>
+      <c r="G1361" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1361" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-15 14:16:02 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1361"/>
+  <dimension ref="A1:H1362"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44407,6 +44407,38 @@
       </c>
       <c r="H1361" s="1" t="inlineStr"/>
     </row>
+    <row r="1362">
+      <c r="A1362" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-15 14:15:58 UTC</t>
+        </is>
+      </c>
+      <c r="B1362" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-15 19:45:58 IST</t>
+        </is>
+      </c>
+      <c r="C1362" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1362" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1362" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1362" s="1" t="inlineStr"/>
+      <c r="G1362" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1362" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-16 14:04:54 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1363"/>
+  <dimension ref="A1:H1364"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44477,6 +44477,38 @@
         <v>76</v>
       </c>
     </row>
+    <row r="1364">
+      <c r="A1364" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-16 14:04:49 UTC</t>
+        </is>
+      </c>
+      <c r="B1364" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-16 19:34:49 IST</t>
+        </is>
+      </c>
+      <c r="C1364" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1364" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1364" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1364" s="1" t="inlineStr"/>
+      <c r="G1364" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1364" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-17 07:56:45 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1364"/>
+  <dimension ref="A1:H1365"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44509,6 +44509,38 @@
       </c>
       <c r="H1364" s="1" t="inlineStr"/>
     </row>
+    <row r="1365">
+      <c r="A1365" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17 07:56:41 UTC</t>
+        </is>
+      </c>
+      <c r="B1365" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:26:41 IST</t>
+        </is>
+      </c>
+      <c r="C1365" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1365" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1365" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1365" s="1" t="inlineStr"/>
+      <c r="G1365" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1365" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-17 13:04:19 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1365"/>
+  <dimension ref="A1:H1366"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44541,6 +44541,38 @@
       </c>
       <c r="H1365" s="1" t="inlineStr"/>
     </row>
+    <row r="1366">
+      <c r="A1366" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:04:14 UTC</t>
+        </is>
+      </c>
+      <c r="B1366" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17 18:34:14 IST</t>
+        </is>
+      </c>
+      <c r="C1366" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1366" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1366" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1366" s="1" t="inlineStr"/>
+      <c r="G1366" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1366" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-18 08:12:21 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1366"/>
+  <dimension ref="A1:H1367"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44573,6 +44573,38 @@
       </c>
       <c r="H1366" s="1" t="inlineStr"/>
     </row>
+    <row r="1367">
+      <c r="A1367" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-18 08:12:16 UTC</t>
+        </is>
+      </c>
+      <c r="B1367" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-18 13:42:16 IST</t>
+        </is>
+      </c>
+      <c r="C1367" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1367" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1367" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1367" s="1" t="inlineStr"/>
+      <c r="G1367" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1367" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-18 13:23:59 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1367"/>
+  <dimension ref="A1:H1368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44605,6 +44605,38 @@
       </c>
       <c r="H1367" s="1" t="inlineStr"/>
     </row>
+    <row r="1368">
+      <c r="A1368" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-18 13:23:56 UTC</t>
+        </is>
+      </c>
+      <c r="B1368" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-18 18:53:56 IST</t>
+        </is>
+      </c>
+      <c r="C1368" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1368" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1368" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1368" s="1" t="inlineStr"/>
+      <c r="G1368" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1368" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-19 09:09:32 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1368"/>
+  <dimension ref="A1:H1369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44637,6 +44637,38 @@
       </c>
       <c r="H1368" s="1" t="inlineStr"/>
     </row>
+    <row r="1369">
+      <c r="A1369" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-19 09:09:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1369" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-19 14:39:27 IST</t>
+        </is>
+      </c>
+      <c r="C1369" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1369" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1369" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1369" s="1" t="inlineStr"/>
+      <c r="G1369" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1369" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-19 16:33:57 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1369"/>
+  <dimension ref="A1:H1370"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44669,6 +44669,38 @@
       </c>
       <c r="H1369" s="1" t="inlineStr"/>
     </row>
+    <row r="1370">
+      <c r="A1370" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-19 16:33:51 UTC</t>
+        </is>
+      </c>
+      <c r="B1370" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-19 22:03:51 IST</t>
+        </is>
+      </c>
+      <c r="C1370" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1370" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1370" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1370" s="1" t="inlineStr"/>
+      <c r="G1370" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1370" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-20 08:45:00 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1370"/>
+  <dimension ref="A1:H1371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44701,6 +44701,38 @@
       </c>
       <c r="H1370" s="1" t="inlineStr"/>
     </row>
+    <row r="1371">
+      <c r="A1371" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-20 08:44:54 UTC</t>
+        </is>
+      </c>
+      <c r="B1371" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-20 14:14:54 IST</t>
+        </is>
+      </c>
+      <c r="C1371" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1371" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1371" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1371" s="1" t="inlineStr"/>
+      <c r="G1371" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1371" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-20 14:24:08 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1371"/>
+  <dimension ref="A1:H1372"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44733,6 +44733,38 @@
       </c>
       <c r="H1371" s="1" t="inlineStr"/>
     </row>
+    <row r="1372">
+      <c r="A1372" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-20 14:24:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1372" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:54:03 IST</t>
+        </is>
+      </c>
+      <c r="C1372" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1372" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1372" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1372" s="1" t="inlineStr"/>
+      <c r="G1372" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1372" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-21 08:45:22 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1372"/>
+  <dimension ref="A1:H1373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44765,6 +44765,38 @@
       </c>
       <c r="H1372" s="1" t="inlineStr"/>
     </row>
+    <row r="1373">
+      <c r="A1373" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:45:18 UTC</t>
+        </is>
+      </c>
+      <c r="B1373" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21 14:15:18 IST</t>
+        </is>
+      </c>
+      <c r="C1373" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1373" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1373" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1373" s="1" t="inlineStr"/>
+      <c r="G1373" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1373" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-21 14:33:22 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1373"/>
+  <dimension ref="A1:H1374"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44797,6 +44797,38 @@
       </c>
       <c r="H1373" s="1" t="inlineStr"/>
     </row>
+    <row r="1374">
+      <c r="A1374" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21 14:33:18 UTC</t>
+        </is>
+      </c>
+      <c r="B1374" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21 20:03:18 IST</t>
+        </is>
+      </c>
+      <c r="C1374" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1374" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1374" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1374" s="1" t="inlineStr"/>
+      <c r="G1374" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1374" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-22 08:47:40 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1374"/>
+  <dimension ref="A1:H1375"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44829,6 +44829,38 @@
       </c>
       <c r="H1374" s="1" t="inlineStr"/>
     </row>
+    <row r="1375">
+      <c r="A1375" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:47:35 UTC</t>
+        </is>
+      </c>
+      <c r="B1375" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:17:35 IST</t>
+        </is>
+      </c>
+      <c r="C1375" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1375" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1375" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1375" s="1" t="inlineStr"/>
+      <c r="G1375" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1375" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-22 14:35:05 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1375"/>
+  <dimension ref="A1:H1376"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44861,6 +44861,38 @@
       </c>
       <c r="H1375" s="1" t="inlineStr"/>
     </row>
+    <row r="1376">
+      <c r="A1376" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:35:00 UTC</t>
+        </is>
+      </c>
+      <c r="B1376" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-22 20:05:00 IST</t>
+        </is>
+      </c>
+      <c r="C1376" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1376" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1376" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1376" s="1" t="inlineStr"/>
+      <c r="G1376" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1376" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-23 08:43:28 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1376"/>
+  <dimension ref="A1:H1377"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44893,6 +44893,38 @@
       </c>
       <c r="H1376" s="1" t="inlineStr"/>
     </row>
+    <row r="1377">
+      <c r="A1377" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-23 08:43:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1377" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-23 14:13:25 IST</t>
+        </is>
+      </c>
+      <c r="C1377" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1377" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1377" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1377" s="1" t="inlineStr"/>
+      <c r="G1377" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1377" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-23 14:19:21 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1377"/>
+  <dimension ref="A1:H1378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44925,6 +44925,38 @@
       </c>
       <c r="H1377" s="1" t="inlineStr"/>
     </row>
+    <row r="1378">
+      <c r="A1378" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-23 14:19:16 UTC</t>
+        </is>
+      </c>
+      <c r="B1378" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-23 19:49:16 IST</t>
+        </is>
+      </c>
+      <c r="C1378" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1378" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1378" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1378" s="1" t="inlineStr"/>
+      <c r="G1378" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1378" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-24 13:26:20 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1379"/>
+  <dimension ref="A1:H1380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -44995,6 +44995,38 @@
         <v>77</v>
       </c>
     </row>
+    <row r="1380">
+      <c r="A1380" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-24 13:26:17 UTC</t>
+        </is>
+      </c>
+      <c r="B1380" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-24 18:56:17 IST</t>
+        </is>
+      </c>
+      <c r="C1380" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1380" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1380" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1380" s="1" t="inlineStr"/>
+      <c r="G1380" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1380" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-25 08:36:12 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1380"/>
+  <dimension ref="A1:H1381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -45027,6 +45027,38 @@
       </c>
       <c r="H1380" s="1" t="inlineStr"/>
     </row>
+    <row r="1381">
+      <c r="A1381" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-25 08:36:07 UTC</t>
+        </is>
+      </c>
+      <c r="B1381" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-25 14:06:07 IST</t>
+        </is>
+      </c>
+      <c r="C1381" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1381" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1381" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1381" s="1" t="inlineStr"/>
+      <c r="G1381" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1381" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-25 13:48:10 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1381"/>
+  <dimension ref="A1:H1382"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -45059,6 +45059,38 @@
       </c>
       <c r="H1381" s="1" t="inlineStr"/>
     </row>
+    <row r="1382">
+      <c r="A1382" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-25 13:48:06 UTC</t>
+        </is>
+      </c>
+      <c r="B1382" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-25 19:18:06 IST</t>
+        </is>
+      </c>
+      <c r="C1382" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1382" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1382" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1382" s="1" t="inlineStr"/>
+      <c r="G1382" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1382" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-26 09:12:28 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1382"/>
+  <dimension ref="A1:H1383"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -45091,6 +45091,38 @@
       </c>
       <c r="H1382" s="1" t="inlineStr"/>
     </row>
+    <row r="1383">
+      <c r="A1383" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-26 09:12:23 UTC</t>
+        </is>
+      </c>
+      <c r="B1383" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-26 14:42:23 IST</t>
+        </is>
+      </c>
+      <c r="C1383" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1383" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1383" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1383" s="1" t="inlineStr"/>
+      <c r="G1383" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1383" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-26 16:13:49 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1383"/>
+  <dimension ref="A1:H1384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -45123,6 +45123,38 @@
       </c>
       <c r="H1383" s="1" t="inlineStr"/>
     </row>
+    <row r="1384">
+      <c r="A1384" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-26 16:13:44 UTC</t>
+        </is>
+      </c>
+      <c r="B1384" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-26 21:43:44 IST</t>
+        </is>
+      </c>
+      <c r="C1384" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1384" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1384" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1384" s="1" t="inlineStr"/>
+      <c r="G1384" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1384" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-27 09:13:04 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1384"/>
+  <dimension ref="A1:H1385"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -45155,6 +45155,38 @@
       </c>
       <c r="H1384" s="1" t="inlineStr"/>
     </row>
+    <row r="1385">
+      <c r="A1385" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-27 09:12:58 UTC</t>
+        </is>
+      </c>
+      <c r="B1385" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-27 14:42:58 IST</t>
+        </is>
+      </c>
+      <c r="C1385" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1385" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1385" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1385" s="1" t="inlineStr"/>
+      <c r="G1385" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1385" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-27 15:27:55 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1385"/>
+  <dimension ref="A1:H1386"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -45187,6 +45187,38 @@
       </c>
       <c r="H1385" s="1" t="inlineStr"/>
     </row>
+    <row r="1386">
+      <c r="A1386" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-27 15:27:50 UTC</t>
+        </is>
+      </c>
+      <c r="B1386" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-27 20:57:50 IST</t>
+        </is>
+      </c>
+      <c r="C1386" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1386" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1386" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1386" s="1" t="inlineStr"/>
+      <c r="G1386" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1386" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-28 09:54:14 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1386"/>
+  <dimension ref="A1:H1387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -45219,6 +45219,38 @@
       </c>
       <c r="H1386" s="1" t="inlineStr"/>
     </row>
+    <row r="1387">
+      <c r="A1387" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-28 09:54:09 UTC</t>
+        </is>
+      </c>
+      <c r="B1387" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-28 15:24:09 IST</t>
+        </is>
+      </c>
+      <c r="C1387" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1387" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1387" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1387" s="1" t="inlineStr"/>
+      <c r="G1387" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1387" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-28 18:24:36 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1387"/>
+  <dimension ref="A1:H1388"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -45251,6 +45251,38 @@
       </c>
       <c r="H1387" s="1" t="inlineStr"/>
     </row>
+    <row r="1388">
+      <c r="A1388" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-28 18:24:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1388" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-28 23:54:30 IST</t>
+        </is>
+      </c>
+      <c r="C1388" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1388" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1388" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1388" s="1" t="inlineStr"/>
+      <c r="G1388" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1388" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-29 18:34:24 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1389"/>
+  <dimension ref="A1:H1390"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -45321,6 +45321,38 @@
         <v>78</v>
       </c>
     </row>
+    <row r="1390">
+      <c r="A1390" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-29 18:34:19 UTC</t>
+        </is>
+      </c>
+      <c r="B1390" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-30 00:04:19 IST</t>
+        </is>
+      </c>
+      <c r="C1390" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1390" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1390" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1390" s="1" t="inlineStr"/>
+      <c r="G1390" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1390" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-30 10:18:08 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1390"/>
+  <dimension ref="A1:H1391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -45353,6 +45353,38 @@
       </c>
       <c r="H1390" s="1" t="inlineStr"/>
     </row>
+    <row r="1391">
+      <c r="A1391" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-30 10:18:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1391" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-30 15:48:03 IST</t>
+        </is>
+      </c>
+      <c r="C1391" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1391" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1391" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1391" s="1" t="inlineStr"/>
+      <c r="G1391" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1391" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-30 18:06:44 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1391"/>
+  <dimension ref="A1:H1392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -45385,6 +45385,38 @@
       </c>
       <c r="H1391" s="1" t="inlineStr"/>
     </row>
+    <row r="1392">
+      <c r="A1392" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:06:39 UTC</t>
+        </is>
+      </c>
+      <c r="B1392" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-30 23:36:39 IST</t>
+        </is>
+      </c>
+      <c r="C1392" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1392" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1392" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1392" s="1" t="inlineStr"/>
+      <c r="G1392" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1392" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-31 09:51:11 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1392"/>
+  <dimension ref="A1:H1393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -45417,6 +45417,38 @@
       </c>
       <c r="H1392" s="1" t="inlineStr"/>
     </row>
+    <row r="1393">
+      <c r="A1393" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-31 09:51:08 UTC</t>
+        </is>
+      </c>
+      <c r="B1393" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-31 15:21:08 IST</t>
+        </is>
+      </c>
+      <c r="C1393" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1393" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1393" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1393" s="1" t="inlineStr"/>
+      <c r="G1393" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1393" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-10-31 17:18:03 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1393"/>
+  <dimension ref="A1:H1394"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -45449,6 +45449,38 @@
       </c>
       <c r="H1393" s="1" t="inlineStr"/>
     </row>
+    <row r="1394">
+      <c r="A1394" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-31 17:17:57 UTC</t>
+        </is>
+      </c>
+      <c r="B1394" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-31 22:47:57 IST</t>
+        </is>
+      </c>
+      <c r="C1394" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1394" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Skipping download &amp; Excel update.</t>
+        </is>
+      </c>
+      <c r="E1394" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1394" s="1" t="inlineStr"/>
+      <c r="G1394" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1394" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>